<commit_message>
fix: corrections QA display names SCT et définitions CodeSystems
- SCT#33586001 : "Sitting position" → "position assise"
- SCT#32750006 : "Inspection" → "examen visuel"
- SCT#7569003 : "Finger structure" → "doigt d'une main excepté le pouce"
- CodeSystemv2-3307, TypeChambre, PositionLit : ajout définitions manquantes
- DisciplineEquipement#552 : suppression espace blanc parasite

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> 204390b46c7a36a9a5607a1fe6d0c8b77d72af12
</commit_message>
<xml_diff>
--- a/nr-add-more-examples/ig/CodeSystem-fr-core-cs-discipline-equipement.xlsx
+++ b/nr-add-more-examples/ig/CodeSystem-fr-core-cs-discipline-equipement.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-30T12:46:16+00:00</t>
+    <t>2026-04-30T13:10:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -585,7 +585,7 @@
     <t>552</t>
   </si>
   <si>
-    <t xml:space="preserve">Entraînement à l'hémodialyse </t>
+    <t>Entraînement à l'hémodialyse</t>
   </si>
   <si>
     <t>553</t>

</xml_diff>